<commit_message>
Rename shroud to fairing in all user-facing surfaces; add catalog fairing tab
Terminology: the template section is now FAIRING (with labels Fairing
mass/length/diameter/nose), the Thrusty GUI says Has Fairing, and the
trajectory event/debris labels read Fairing jettison / Fairing impact /
Fairing. Internal keys stay shroud_* so existing saved missiles and JSON
files load unchanged; the XLSX importer is row-number-based, so old and
new workbooks both import.

Catalog format: new 'fairing' tab (one row per model_id: mass_kg,
jettison_alt_km, length_m, diameter_m, nose_shape, nose_length_m) in
make_catalog_template.py, regenerated catalog_template_draft.xlsx, and
the JL-2 catalog now carries its 298 kg / 2 km fairing row.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FYmY1XBusSrATRZ4jAxiDg
</commit_message>
<xml_diff>
--- a/docs/ingestion/catalog_template_draft.xlsx
+++ b/docs/ingestion/catalog_template_draft.xlsx
@@ -9,8 +9,9 @@
   <sheets>
     <sheet name="rockets" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="payloads" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="enums" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="README" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="fairing" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="enums" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="README" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1603,6 +1604,87 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>DRAFT — one row per model with a fairing (keyed by model_id; maps to the shroud_* params). jettison_alt_km: 80 is the launch-vehicle default; SLBM water-egress fairings shed low (~2 km).</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>model_id</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>mass_kg</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>jettison_alt_km</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>length_m</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>diameter_m</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>nose_shape</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>nose_length_m</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>source_citation</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="F3:F400" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"cone,tangent_ogive,von_karman,lv_haack,parabola,blunt_cylinder"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1946,13 +2028,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1971,7 +2053,7 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Two record types live in two tabs:</t>
+          <t>Record types live in their own tabs:</t>
         </is>
       </c>
     </row>
@@ -1990,83 +2072,90 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr"/>
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • fairing  — one row per model with a fairing, keyed by model_id (maps to the shroud_* params).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Conventions</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • BLANK numeric cells are intentional — the ingest resolver estimates them and flags VERIFY.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Peach-tinted columns in `rockets` are MODEL-level: fill them once on the stage_no=1 row.</t>
+          <t xml:space="preserve">  • BLANK numeric cells are intentional — the ingest resolver estimates them and flags VERIFY.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • payload_id links a rocket to a payloads row. Leave blank for orbital launches (a</t>
+          <t xml:space="preserve">  • Peach-tinted columns in `rockets` are MODEL-level: fill them once on the stage_no=1 row.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">    satellite is not an RV) and set terminal_mode=orbital + payload_kg instead.</t>
+          <t xml:space="preserve">  • payload_id links a rocket to a payloads row. Leave blank for orbital launches (a</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • marv_body payloads inherit mass/diameter/length from the missile burnout — leave blank.</t>
+          <t xml:space="preserve">    satellite is not an RV) and set terminal_mode=orbital + payload_kg instead.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
+          <t xml:space="preserve">  • marv_body payloads inherit mass/diameter/length from the missile burnout — leave blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">  • solid_motor=YES enables grain_type; guidance=orbital_insertion belongs on the final SLV stage.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="7" t="inlineStr"/>
-    </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
         <is>
           <t>Running in Thrusty</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Live:    File → Share (anyone-with-link viewer), then give Thrusty the sheet URL;</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">             it fetches  …/export?format=xlsx  (both tabs, no auth).</t>
+          <t xml:space="preserve">  • Live:    File → Share (anyone-with-link viewer), then give Thrusty the sheet URL;</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">             it fetches  …/export?format=xlsx  (both tabs, no auth).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">  • Upload:  File → Download → .xlsx  and open the file in Thrusty (same importer).</t>
         </is>

</xml_diff>